<commit_message>
feat: complete Excel engine refactoring, hybrid template generation, and clear-then-write sample data cleaning
- Implemented clear-then-write cell engine logic to prevent template sample data leakage
- Enforced strict VARIABLE vs FIXED cell classification across all worksheets
- Preserved row heights, customHeight properties, and layout dimensions across hybrid master templates
- Added automatic breaker sheet pruning when has_breaker is false
- Removed self-registration and obsolete user profile fields (Sicil, EKIPNET, Diploma)
- Added missing breaker measurement fields to report creation form
- Verified T1, T2, T3 acceptance tests with 100% pass rate and 0 Excel repair warnings
</commit_message>
<xml_diff>
--- a/backend/templates/hybrid/gt_hybrid.xlsx
+++ b/backend/templates/hybrid/gt_hybrid.xlsx
@@ -5270,89 +5270,6 @@
   </twoCellAnchor>
   <twoCellAnchor editAs="oneCell">
     <from>
-      <col>6</col>
-      <colOff>28574</colOff>
-      <row>52</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <to>
-      <col>11</col>
-      <colOff>1444</colOff>
-      <row>55</row>
-      <rowOff>19050</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Resim 11"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r="62" b="55405"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3038474" y="9344025"/>
-          <a:ext cx="2316020" cy="561975"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>11</col>
-      <colOff>38100</colOff>
-      <row>52</row>
-      <rowOff>123825</rowOff>
-    </from>
-    <to>
-      <col>12</col>
-      <colOff>549564</colOff>
-      <row>54</row>
-      <rowOff>177827</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Resim 12"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5391150" y="9439275"/>
-          <a:ext cx="1121064" cy="435003"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
       <col>10</col>
       <colOff>0</colOff>
       <row>1</row>
@@ -5372,7 +5289,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -5413,7 +5330,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" b="4827"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -5455,7 +5372,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" b="8860"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -5465,48 +5382,6 @@
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="5969870" y="207754"/>
           <a:ext cx="581977" cy="432093"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>31</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>6</col>
-      <colOff>420896</colOff>
-      <row>50</row>
-      <rowOff>134327</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Resim 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="37248" t="22100" r="38025" b="30578"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="5238750"/>
-          <a:ext cx="3437146" cy="3700096"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
@@ -5565,88 +5440,6 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>76199</colOff>
-      <row>50</row>
-      <rowOff>38100</rowOff>
-    </from>
-    <to>
-      <col>13</col>
-      <colOff>96900</colOff>
-      <row>52</row>
-      <rowOff>238125</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Resim 5"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3209924" y="9324975"/>
-          <a:ext cx="1468501" cy="771525"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>12</col>
-      <colOff>209550</colOff>
-      <row>51</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>313181</colOff>
-      <row>52</row>
-      <rowOff>85028</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Resim 4"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="4429125" y="9572625"/>
-          <a:ext cx="1551431" cy="370778"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -5683,88 +5476,6 @@
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="235324" y="190500"/>
           <a:ext cx="1819275" cy="745435"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>59908</colOff>
-      <row>48</row>
-      <rowOff>18531</rowOff>
-    </from>
-    <to>
-      <col>13</col>
-      <colOff>203902</colOff>
-      <row>50</row>
-      <rowOff>265061</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Resim 8"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3173850" y="9360358"/>
-          <a:ext cx="1580071" cy="818030"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>12</col>
-      <colOff>124556</colOff>
-      <row>48</row>
-      <rowOff>249116</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>239910</colOff>
-      <row>50</row>
-      <rowOff>48394</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Resim 6"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="4315556" y="9590943"/>
-          <a:ext cx="1551431" cy="370778"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
@@ -5823,88 +5534,6 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>57150</colOff>
-      <row>52</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <to>
-      <col>13</col>
-      <colOff>189421</colOff>
-      <row>54</row>
-      <rowOff>275105</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Resim 7"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3143250" y="9229725"/>
-          <a:ext cx="1580071" cy="818030"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>13</col>
-      <colOff>28575</colOff>
-      <row>52</row>
-      <rowOff>238125</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>65531</colOff>
-      <row>54</row>
-      <rowOff>37403</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Resim 5"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="4562475" y="9439275"/>
-          <a:ext cx="1551431" cy="370778"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -5952,89 +5581,6 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>47624</colOff>
-      <row>52</row>
-      <rowOff>66674</rowOff>
-    </from>
-    <to>
-      <col>15</col>
-      <colOff>154195</colOff>
-      <row>54</row>
-      <rowOff>57149</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Resim 5"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r="4040" b="56470"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3133724" y="9248774"/>
-          <a:ext cx="2278271" cy="561975"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>14</col>
-      <colOff>114300</colOff>
-      <row>52</row>
-      <rowOff>247650</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>82839</colOff>
-      <row>54</row>
-      <rowOff>111153</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Resim 6"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5010150" y="9429750"/>
-          <a:ext cx="1121064" cy="435003"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -6071,89 +5617,6 @@
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="107674" y="66261"/>
           <a:ext cx="2017125" cy="745435"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>10</col>
-      <colOff>81308</colOff>
-      <row>78</row>
-      <rowOff>46463</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>234322</colOff>
-      <row>80</row>
-      <rowOff>162621</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Resim 6"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r="-1725" b="54025"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3217588" y="9257835"/>
-          <a:ext cx="2174173" cy="534329"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>15</col>
-      <colOff>209086</colOff>
-      <row>79</row>
-      <rowOff>11617</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>319570</colOff>
-      <row>81</row>
-      <rowOff>28449</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Resim 3"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5029665" y="9432074"/>
-          <a:ext cx="1121064" cy="435003"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
@@ -6239,89 +5702,6 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>28574</colOff>
-      <row>45</row>
-      <rowOff>190499</rowOff>
-    </from>
-    <to>
-      <col>14</col>
-      <colOff>73819</colOff>
-      <row>47</row>
-      <rowOff>104774</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Resim 9"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" t="-1" r="2758" b="54343"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3238499" y="9467849"/>
-          <a:ext cx="1902620" cy="485775"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>14</col>
-      <colOff>28575</colOff>
-      <row>45</row>
-      <rowOff>180975</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>35214</colOff>
-      <row>47</row>
-      <rowOff>44478</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Resim 10"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5095875" y="9458325"/>
-          <a:ext cx="1121064" cy="435003"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -6385,89 +5765,6 @@
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="238125" y="190500"/>
           <a:ext cx="1885950" cy="745435"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>57149</colOff>
-      <row>45</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>14</col>
-      <colOff>268381</colOff>
-      <row>46</row>
-      <rowOff>257175</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Resim 8"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r="3480" b="57500"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3267074" y="9324975"/>
-          <a:ext cx="2068607" cy="495300"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>14</col>
-      <colOff>47625</colOff>
-      <row>45</row>
-      <rowOff>171450</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>54264</colOff>
-      <row>47</row>
-      <rowOff>34953</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Resim 10"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5114925" y="9448800"/>
-          <a:ext cx="1121064" cy="435003"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
@@ -6607,89 +5904,6 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>67234</colOff>
-      <row>50</row>
-      <rowOff>123265</rowOff>
-    </from>
-    <to>
-      <col>14</col>
-      <colOff>67238</colOff>
-      <row>52</row>
-      <rowOff>78441</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Resim 10"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r="5512" b="56559"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3518646" y="10208559"/>
-          <a:ext cx="2151533" cy="537882"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>14</col>
-      <colOff>89648</colOff>
-      <row>50</row>
-      <rowOff>246530</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>392682</colOff>
-      <row>52</row>
-      <rowOff>98827</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Resim 12"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5692589" y="10331824"/>
-          <a:ext cx="1121064" cy="435003"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -6764,89 +5978,6 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>33617</colOff>
-      <row>50</row>
-      <rowOff>212911</rowOff>
-    </from>
-    <to>
-      <col>13</col>
-      <colOff>358589</colOff>
-      <row>52</row>
-      <rowOff>67234</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Resim 7"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" t="1" r="-988" b="57143"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3216088" y="10286999"/>
-          <a:ext cx="1893795" cy="437029"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>13</col>
-      <colOff>369794</colOff>
-      <row>50</row>
-      <rowOff>224118</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>280623</colOff>
-      <row>52</row>
-      <rowOff>76415</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Resim 8"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5121088" y="10298206"/>
-          <a:ext cx="1121064" cy="435003"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -6883,88 +6014,6 @@
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="235323" y="190500"/>
           <a:ext cx="1748117" cy="745435"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>179294</colOff>
-      <row>47</row>
-      <rowOff>44824</rowOff>
-    </from>
-    <to>
-      <col>13</col>
-      <colOff>213483</colOff>
-      <row>49</row>
-      <rowOff>263101</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Resim 7"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3193676" y="9379324"/>
-          <a:ext cx="1524572" cy="800983"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>13</col>
-      <colOff>56029</colOff>
-      <row>47</row>
-      <rowOff>246529</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>38637</colOff>
-      <row>49</row>
-      <rowOff>34601</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Resim 6"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="4560794" y="9581029"/>
-          <a:ext cx="1551431" cy="370778"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
@@ -7023,88 +6072,6 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>10</col>
-      <colOff>95250</colOff>
-      <row>74</row>
-      <rowOff>19050</rowOff>
-    </from>
-    <to>
-      <col>13</col>
-      <colOff>266700</colOff>
-      <row>77</row>
-      <rowOff>120225</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Resim 5"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3200400" y="9448800"/>
-          <a:ext cx="1171575" cy="615525"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>13</col>
-      <colOff>190500</colOff>
-      <row>75</row>
-      <rowOff>19050</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>75056</colOff>
-      <row>77</row>
-      <rowOff>46928</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Resim 4"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="4295775" y="9620250"/>
-          <a:ext cx="1551431" cy="370778"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -7141,88 +6108,6 @@
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="238125" y="190500"/>
           <a:ext cx="1819275" cy="745435"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>9</col>
-      <colOff>190500</colOff>
-      <row>50</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>13</col>
-      <colOff>174942</colOff>
-      <row>52</row>
-      <rowOff>228600</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Resim 8"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="3324225" y="9324975"/>
-          <a:ext cx="1432242" cy="752475"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>12</col>
-      <colOff>190500</colOff>
-      <row>50</row>
-      <rowOff>247650</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>27431</colOff>
-      <row>52</row>
-      <rowOff>46928</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Resim 6"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="4410075" y="9525000"/>
-          <a:ext cx="1551431" cy="370778"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
@@ -8011,7 +6896,7 @@
     <col width="9.109375" customWidth="1" style="227" min="19" max="19"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="15" customHeight="1" s="227">
       <c r="A1" s="12" t="n"/>
       <c r="B1" s="13" t="n"/>
       <c r="C1" s="13" t="n"/>
@@ -8224,7 +7109,7 @@
       <c r="Q9" s="143" t="n"/>
       <c r="R9" s="11" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="15" customHeight="1" s="227">
       <c r="A10" s="10" t="n"/>
       <c r="B10" s="421" t="inlineStr">
         <is>
@@ -8232,11 +7117,7 @@
         </is>
       </c>
       <c r="C10" s="482" t="n"/>
-      <c r="D10" s="422" t="inlineStr">
-        <is>
-          <t>Hilmi GÜL</t>
-        </is>
-      </c>
+      <c r="D10" s="422" t="n"/>
       <c r="E10" s="99" t="n"/>
       <c r="F10" s="99" t="n"/>
       <c r="G10" s="482" t="n"/>
@@ -8246,11 +7127,7 @@
         </is>
       </c>
       <c r="I10" s="482" t="n"/>
-      <c r="J10" s="374" t="inlineStr">
-        <is>
-          <t>STS 5000</t>
-        </is>
-      </c>
+      <c r="J10" s="374" t="n"/>
       <c r="K10" s="99" t="n"/>
       <c r="L10" s="482" t="n"/>
       <c r="M10" s="374" t="inlineStr">
@@ -8259,11 +7136,7 @@
         </is>
       </c>
       <c r="N10" s="482" t="n"/>
-      <c r="O10" s="374" t="inlineStr">
-        <is>
-          <t>19B20</t>
-        </is>
-      </c>
+      <c r="O10" s="374" t="n"/>
       <c r="P10" s="99" t="n"/>
       <c r="Q10" s="482" t="n"/>
       <c r="R10" s="11" t="n"/>
@@ -8383,7 +7256,7 @@
       <c r="Q15" s="41" t="n"/>
       <c r="R15" s="11" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="15" customHeight="1" s="227">
       <c r="A16" s="10" t="n"/>
       <c r="B16" s="384" t="inlineStr">
         <is>
@@ -8400,7 +7273,7 @@
       <c r="Q16" s="212" t="n"/>
       <c r="R16" s="11" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="15" customHeight="1" s="227">
       <c r="A17" s="10" t="n"/>
       <c r="B17" s="377" t="inlineStr">
         <is>
@@ -8432,7 +7305,7 @@
       <c r="Q17" s="212" t="n"/>
       <c r="R17" s="11" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" ht="15" customHeight="1" s="227">
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="377" t="n"/>
       <c r="F18" s="446" t="n"/>
@@ -8453,7 +7326,7 @@
       <c r="Q18" s="212" t="n"/>
       <c r="R18" s="11" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="15" customHeight="1" s="227">
       <c r="A19" s="10" t="n"/>
       <c r="B19" s="377" t="inlineStr">
         <is>
@@ -8476,7 +7349,7 @@
       <c r="Q19" s="212" t="n"/>
       <c r="R19" s="11" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" ht="15" customHeight="1" s="227">
       <c r="A20" s="10" t="n"/>
       <c r="B20" s="302" t="inlineStr">
         <is>
@@ -8579,7 +7452,7 @@
       <c r="Q23" s="482" t="n"/>
       <c r="R23" s="11" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" ht="15" customHeight="1" s="227">
       <c r="A24" s="10" t="n"/>
       <c r="B24" s="39" t="n"/>
       <c r="C24" s="40" t="n"/>
@@ -8604,7 +7477,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="15" customHeight="1" s="227">
       <c r="A25" s="10" t="n"/>
       <c r="B25" s="384" t="inlineStr">
         <is>
@@ -8627,7 +7500,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="15" customHeight="1" s="227">
       <c r="A26" s="10" t="n"/>
       <c r="B26" s="377" t="inlineStr">
         <is>
@@ -8664,7 +7537,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="15" customHeight="1" s="227">
       <c r="A27" s="10" t="n"/>
       <c r="B27" s="377" t="n"/>
       <c r="F27" s="446" t="n"/>
@@ -8690,7 +7563,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="15" customHeight="1" s="227">
       <c r="A28" s="10" t="n"/>
       <c r="B28" s="377" t="inlineStr">
         <is>
@@ -8718,7 +7591,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="15" customHeight="1" s="227">
       <c r="A29" s="10" t="n"/>
       <c r="B29" s="302" t="inlineStr">
         <is>
@@ -8829,7 +7702,7 @@
       <c r="Q32" s="482" t="n"/>
       <c r="R32" s="11" t="n"/>
     </row>
-    <row r="33">
+    <row r="33" ht="15" customHeight="1" s="227">
       <c r="A33" s="10" t="n"/>
       <c r="B33" s="39" t="n"/>
       <c r="C33" s="40" t="n"/>
@@ -8849,7 +7722,7 @@
       <c r="Q33" s="41" t="n"/>
       <c r="R33" s="11" t="n"/>
     </row>
-    <row r="34">
+    <row r="34" ht="15" customHeight="1" s="227">
       <c r="A34" s="10" t="n"/>
       <c r="B34" s="384" t="inlineStr">
         <is>
@@ -8867,7 +7740,7 @@
       <c r="Q34" s="212" t="n"/>
       <c r="R34" s="11" t="n"/>
     </row>
-    <row r="35">
+    <row r="35" ht="15" customHeight="1" s="227">
       <c r="A35" s="10" t="n"/>
       <c r="B35" s="377" t="inlineStr">
         <is>
@@ -8899,7 +7772,7 @@
       <c r="Q35" s="212" t="n"/>
       <c r="R35" s="11" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="15" customHeight="1" s="227">
       <c r="A36" s="10" t="n"/>
       <c r="B36" s="377" t="n"/>
       <c r="F36" s="446" t="n"/>
@@ -9327,8 +8200,8 @@
     <mergeCell ref="M10:N10"/>
     <mergeCell ref="F16:I16"/>
     <mergeCell ref="F25:I25"/>
+    <mergeCell ref="N39:O39"/>
     <mergeCell ref="B8:I8"/>
-    <mergeCell ref="N39:O39"/>
     <mergeCell ref="J19:M19"/>
     <mergeCell ref="P39:Q39"/>
     <mergeCell ref="J28:M28"/>
@@ -9464,7 +8337,7 @@
     <col width="9.109375" customWidth="1" style="227" min="19" max="19"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="15" customHeight="1" s="227">
       <c r="A1" s="12" t="n"/>
       <c r="B1" s="13" t="n"/>
       <c r="C1" s="13" t="n"/>
@@ -9660,7 +8533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="15" customHeight="1" s="227">
       <c r="A9" s="10" t="n"/>
       <c r="B9" s="421" t="inlineStr">
         <is>
@@ -9681,11 +8554,7 @@
         </is>
       </c>
       <c r="I9" s="482" t="n"/>
-      <c r="J9" s="374" t="inlineStr">
-        <is>
-          <t>METREL MI 3210</t>
-        </is>
-      </c>
+      <c r="J9" s="374" t="n"/>
       <c r="K9" s="99" t="n"/>
       <c r="L9" s="482" t="n"/>
       <c r="M9" s="374" t="inlineStr">
@@ -9694,9 +8563,7 @@
         </is>
       </c>
       <c r="N9" s="482" t="n"/>
-      <c r="O9" s="374" t="n">
-        <v>16060016</v>
-      </c>
+      <c r="O9" s="374" t="n"/>
       <c r="P9" s="99" t="n"/>
       <c r="Q9" s="482" t="n"/>
       <c r="R9" s="11" t="n"/>
@@ -10149,7 +9016,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="15" customHeight="1" s="227">
       <c r="A25" s="33" t="n"/>
       <c r="B25" s="398" t="inlineStr">
         <is>
@@ -10217,7 +9084,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="15" customHeight="1" s="227">
       <c r="A26" s="33" t="n"/>
       <c r="B26" s="398" t="inlineStr">
         <is>
@@ -10259,7 +9126,7 @@
       <c r="Q26" s="213" t="n"/>
       <c r="R26" s="11" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="15" customHeight="1" s="227">
       <c r="A27" s="33" t="n"/>
       <c r="B27" s="398" t="inlineStr">
         <is>
@@ -10323,7 +9190,7 @@
       </c>
       <c r="R27" s="11" t="n"/>
     </row>
-    <row r="28">
+    <row r="28" ht="15" customHeight="1" s="227">
       <c r="A28" s="33" t="n"/>
       <c r="B28" s="627" t="inlineStr">
         <is>
@@ -10442,7 +9309,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="15" customHeight="1" s="227">
       <c r="A32" s="10" t="n"/>
       <c r="B32" s="3" t="n"/>
       <c r="C32" s="127" t="n"/>
@@ -10461,7 +9328,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="15" customHeight="1" s="227">
       <c r="A33" s="10" t="n"/>
       <c r="B33" s="3" t="n"/>
       <c r="C33" s="127" t="n"/>
@@ -10480,7 +9347,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="15" customHeight="1" s="227">
       <c r="A34" s="10" t="n"/>
       <c r="B34" s="24" t="n"/>
       <c r="C34" s="25" t="n"/>
@@ -10500,7 +9367,7 @@
       <c r="Q34" s="143" t="n"/>
       <c r="R34" s="11" t="n"/>
     </row>
-    <row r="35">
+    <row r="35" ht="15" customHeight="1" s="227">
       <c r="A35" s="10" t="n"/>
       <c r="B35" s="3" t="n"/>
       <c r="C35" s="127" t="n"/>
@@ -10520,7 +9387,7 @@
       <c r="Q35" s="143" t="n"/>
       <c r="R35" s="11" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="15" customHeight="1" s="227">
       <c r="A36" s="10" t="n"/>
       <c r="B36" s="3" t="n"/>
       <c r="C36" s="127" t="n"/>
@@ -10882,34 +9749,34 @@
       <c r="Q52" s="16" t="n"/>
       <c r="R52" s="17" t="n"/>
     </row>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
+    <row r="53" ht="15" customHeight="1" s="227"/>
+    <row r="54" ht="15" customHeight="1" s="227"/>
+    <row r="55" ht="15" customHeight="1" s="227"/>
     <row r="56" ht="18" customHeight="1" s="227">
       <c r="S56" s="54" t="n"/>
     </row>
-    <row r="57">
+    <row r="57" ht="15" customHeight="1" s="227">
       <c r="S57" s="127" t="n"/>
     </row>
-    <row r="58">
+    <row r="58" ht="15" customHeight="1" s="227">
       <c r="S58" s="27" t="n"/>
     </row>
-    <row r="59">
+    <row r="59" ht="15" customHeight="1" s="227">
       <c r="S59" s="127" t="n"/>
     </row>
-    <row r="60">
+    <row r="60" ht="15" customHeight="1" s="227">
       <c r="S60" s="635" t="n"/>
     </row>
-    <row r="61">
+    <row r="61" ht="15" customHeight="1" s="227">
       <c r="S61" s="127" t="n"/>
     </row>
-    <row r="62">
+    <row r="62" ht="15" customHeight="1" s="227">
       <c r="S62" s="127" t="n"/>
     </row>
-    <row r="63">
+    <row r="63" ht="15" customHeight="1" s="227">
       <c r="S63" s="127" t="n"/>
     </row>
-    <row r="64">
+    <row r="64" ht="15" customHeight="1" s="227">
       <c r="S64" s="127" t="n"/>
     </row>
   </sheetData>
@@ -10981,8 +9848,8 @@
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="J9:L9"/>
     <mergeCell ref="B28:E28"/>
+    <mergeCell ref="I27:I28"/>
     <mergeCell ref="W38:AJ38"/>
-    <mergeCell ref="I27:I28"/>
     <mergeCell ref="J23:Q23"/>
     <mergeCell ref="W28:AD28"/>
     <mergeCell ref="N19:Q19"/>
@@ -11185,7 +10052,7 @@
       <c r="Q6" s="143" t="n"/>
       <c r="R6" s="11" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="15" customHeight="1" s="227">
       <c r="A7" s="10" t="n"/>
       <c r="B7" s="421" t="inlineStr">
         <is>
@@ -11226,7 +10093,7 @@
       <c r="Q7" s="482" t="n"/>
       <c r="R7" s="11" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="15" customHeight="1" s="227">
       <c r="A8" s="10" t="n"/>
       <c r="B8" s="374" t="inlineStr">
         <is>
@@ -11809,7 +10676,7 @@
       <c r="Q31" s="652" t="n"/>
       <c r="R31" s="11" t="n"/>
     </row>
-    <row r="32">
+    <row r="32" ht="15" customHeight="1" s="227">
       <c r="A32" s="10" t="n"/>
       <c r="B32" s="422" t="inlineStr">
         <is>
@@ -11925,7 +10792,7 @@
       <c r="Q35" s="655" t="n"/>
       <c r="R35" s="11" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="15" customHeight="1" s="227">
       <c r="A36" s="10" t="n"/>
       <c r="B36" s="422" t="inlineStr">
         <is>
@@ -11984,7 +10851,7 @@
       <c r="Q37" s="659" t="n"/>
       <c r="R37" s="11" t="n"/>
     </row>
-    <row r="38">
+    <row r="38" ht="15" customHeight="1" s="227">
       <c r="A38" s="10" t="n"/>
       <c r="B38" s="656" t="inlineStr">
         <is>
@@ -12022,7 +10889,7 @@
       <c r="Q39" s="212" t="n"/>
       <c r="R39" s="11" t="n"/>
     </row>
-    <row r="40">
+    <row r="40" ht="15" customHeight="1" s="227">
       <c r="A40" s="10" t="n"/>
       <c r="B40" s="3" t="n"/>
       <c r="C40" s="317" t="inlineStr">
@@ -12044,7 +10911,7 @@
       <c r="Q41" s="55" t="n"/>
       <c r="R41" s="11" t="n"/>
     </row>
-    <row r="42">
+    <row r="42" ht="15" customHeight="1" s="227">
       <c r="A42" s="10" t="n"/>
       <c r="B42" s="3" t="n"/>
       <c r="C42" s="317" t="inlineStr">
@@ -12055,7 +10922,7 @@
       <c r="Q42" s="143" t="n"/>
       <c r="R42" s="11" t="n"/>
     </row>
-    <row r="43">
+    <row r="43" ht="15" customHeight="1" s="227">
       <c r="A43" s="10" t="n"/>
       <c r="B43" s="528" t="n"/>
       <c r="C43" s="317" t="inlineStr">
@@ -12066,7 +10933,7 @@
       <c r="Q43" s="143" t="n"/>
       <c r="R43" s="11" t="n"/>
     </row>
-    <row r="44">
+    <row r="44" ht="15" customHeight="1" s="227">
       <c r="A44" s="10" t="n"/>
       <c r="B44" s="528" t="n"/>
       <c r="C44" s="317" t="inlineStr">
@@ -12077,7 +10944,7 @@
       <c r="Q44" s="117" t="n"/>
       <c r="R44" s="11" t="n"/>
     </row>
-    <row r="45">
+    <row r="45" ht="15" customHeight="1" s="227">
       <c r="A45" s="10" t="n"/>
       <c r="B45" s="528" t="n"/>
       <c r="C45" s="317" t="inlineStr">
@@ -12088,7 +10955,7 @@
       <c r="Q45" s="117" t="n"/>
       <c r="R45" s="11" t="n"/>
     </row>
-    <row r="46">
+    <row r="46" ht="15" customHeight="1" s="227">
       <c r="A46" s="10" t="n"/>
       <c r="B46" s="310" t="n"/>
       <c r="C46" s="662" t="inlineStr">
@@ -12154,7 +11021,7 @@
       <c r="Q50" s="212" t="n"/>
       <c r="R50" s="11" t="n"/>
     </row>
-    <row r="51">
+    <row r="51" ht="15" customHeight="1" s="227">
       <c r="A51" s="10" t="n"/>
       <c r="B51" s="181" t="inlineStr">
         <is>
@@ -12342,10 +11209,10 @@
     <mergeCell ref="B53:D53"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="B47:Q50"/>
+    <mergeCell ref="C45:P45"/>
     <mergeCell ref="N22:O22"/>
-    <mergeCell ref="C45:P45"/>
+    <mergeCell ref="B34:D34"/>
     <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B34:D34"/>
     <mergeCell ref="N36:Q36"/>
     <mergeCell ref="F53:I53"/>
     <mergeCell ref="I8:K8"/>
@@ -16327,11 +15194,7 @@
         </is>
       </c>
       <c r="C11" s="482" t="n"/>
-      <c r="D11" s="422" t="inlineStr">
-        <is>
-          <t>Hilmi GÜL</t>
-        </is>
-      </c>
+      <c r="D11" s="422" t="n"/>
       <c r="E11" s="99" t="n"/>
       <c r="F11" s="99" t="n"/>
       <c r="G11" s="482" t="n"/>
@@ -16341,11 +15204,7 @@
         </is>
       </c>
       <c r="I11" s="482" t="n"/>
-      <c r="J11" s="374" t="inlineStr">
-        <is>
-          <t>STS 5000</t>
-        </is>
-      </c>
+      <c r="J11" s="374" t="n"/>
       <c r="K11" s="99" t="n"/>
       <c r="L11" s="482" t="n"/>
       <c r="M11" s="374" t="inlineStr">
@@ -16354,11 +15213,7 @@
         </is>
       </c>
       <c r="N11" s="482" t="n"/>
-      <c r="O11" s="374" t="inlineStr">
-        <is>
-          <t>19B20</t>
-        </is>
-      </c>
+      <c r="O11" s="374" t="n"/>
       <c r="P11" s="99" t="n"/>
       <c r="Q11" s="482" t="n"/>
       <c r="R11" s="11" t="n"/>
@@ -16687,9 +15542,7 @@
         <v/>
       </c>
       <c r="H24" s="482" t="n"/>
-      <c r="I24" s="370" t="n">
-        <v>40</v>
-      </c>
+      <c r="I24" s="370" t="n"/>
       <c r="J24" s="482" t="n"/>
       <c r="K24" s="370">
         <f>'ANA SAYFA'!C55</f>
@@ -16742,9 +15595,7 @@
         <v/>
       </c>
       <c r="H25" s="482" t="n"/>
-      <c r="I25" s="370" t="n">
-        <v>40</v>
-      </c>
+      <c r="I25" s="370" t="n"/>
       <c r="J25" s="482" t="n"/>
       <c r="K25" s="370">
         <f>'ANA SAYFA'!C59</f>
@@ -16789,9 +15640,7 @@
         <v/>
       </c>
       <c r="H26" s="482" t="n"/>
-      <c r="I26" s="370" t="n">
-        <v>40</v>
-      </c>
+      <c r="I26" s="370" t="n"/>
       <c r="J26" s="482" t="n"/>
       <c r="K26" s="370">
         <f>'ANA SAYFA'!C57</f>
@@ -17673,11 +16522,7 @@
         </is>
       </c>
       <c r="I11" s="482" t="n"/>
-      <c r="J11" s="374" t="inlineStr">
-        <is>
-          <t>STS 5000</t>
-        </is>
-      </c>
+      <c r="J11" s="374" t="n"/>
       <c r="K11" s="99" t="n"/>
       <c r="L11" s="482" t="n"/>
       <c r="M11" s="374" t="inlineStr">
@@ -17686,11 +16531,7 @@
         </is>
       </c>
       <c r="N11" s="482" t="n"/>
-      <c r="O11" s="374" t="inlineStr">
-        <is>
-          <t>19B20</t>
-        </is>
-      </c>
+      <c r="O11" s="374" t="n"/>
       <c r="P11" s="99" t="n"/>
       <c r="Q11" s="482" t="n"/>
       <c r="R11" s="11" t="n"/>
@@ -18015,9 +16856,7 @@
         <v/>
       </c>
       <c r="H24" s="482" t="n"/>
-      <c r="I24" s="370" t="n">
-        <v>35</v>
-      </c>
+      <c r="I24" s="370" t="n"/>
       <c r="J24" s="482" t="n"/>
       <c r="K24" s="503">
         <f>'ANA SAYFA'!G55</f>
@@ -18070,9 +16909,7 @@
         <v/>
       </c>
       <c r="H25" s="482" t="n"/>
-      <c r="I25" s="370" t="n">
-        <v>35</v>
-      </c>
+      <c r="I25" s="370" t="n"/>
       <c r="J25" s="482" t="n"/>
       <c r="K25" s="503">
         <f>'ANA SAYFA'!G57</f>
@@ -18117,9 +16954,7 @@
         <v/>
       </c>
       <c r="H26" s="482" t="n"/>
-      <c r="I26" s="370" t="n">
-        <v>35</v>
-      </c>
+      <c r="I26" s="370" t="n"/>
       <c r="J26" s="482" t="n"/>
       <c r="K26" s="503">
         <f>'ANA SAYFA'!G59</f>
@@ -19062,11 +17897,7 @@
         </is>
       </c>
       <c r="I11" s="482" t="n"/>
-      <c r="J11" s="422" t="inlineStr">
-        <is>
-          <t>METREL-MI3210</t>
-        </is>
-      </c>
+      <c r="J11" s="422" t="n"/>
       <c r="K11" s="99" t="n"/>
       <c r="L11" s="482" t="n"/>
       <c r="M11" s="374" t="inlineStr">
@@ -19075,9 +17906,7 @@
         </is>
       </c>
       <c r="N11" s="482" t="n"/>
-      <c r="O11" s="374" t="n">
-        <v>16060016</v>
-      </c>
+      <c r="O11" s="374" t="n"/>
       <c r="P11" s="99" t="n"/>
       <c r="Q11" s="482" t="n"/>
       <c r="R11" s="11" t="n"/>
@@ -19260,11 +18089,7 @@
         </is>
       </c>
       <c r="C17" s="482" t="n"/>
-      <c r="D17" s="440" t="inlineStr">
-        <is>
-          <t>45 sn</t>
-        </is>
-      </c>
+      <c r="D17" s="440" t="n"/>
       <c r="E17" s="482" t="n"/>
       <c r="F17" s="440" t="inlineStr">
         <is>
@@ -20859,11 +19684,7 @@
         </is>
       </c>
       <c r="I11" s="482" t="n"/>
-      <c r="J11" s="374" t="inlineStr">
-        <is>
-          <t>STS 5000</t>
-        </is>
-      </c>
+      <c r="J11" s="374" t="n"/>
       <c r="K11" s="99" t="n"/>
       <c r="L11" s="482" t="n"/>
       <c r="M11" s="374" t="inlineStr">
@@ -20872,11 +19693,7 @@
         </is>
       </c>
       <c r="N11" s="482" t="n"/>
-      <c r="O11" s="374" t="inlineStr">
-        <is>
-          <t>19B20</t>
-        </is>
-      </c>
+      <c r="O11" s="374" t="n"/>
       <c r="P11" s="99" t="n"/>
       <c r="Q11" s="482" t="n"/>
       <c r="R11" s="11" t="n"/>
@@ -21030,11 +19847,7 @@
     </row>
     <row r="17">
       <c r="A17" s="10" t="n"/>
-      <c r="B17" s="384" t="inlineStr">
-        <is>
-          <t>Nominal Değerler</t>
-        </is>
-      </c>
+      <c r="B17" s="384" t="n"/>
       <c r="F17" s="446" t="n"/>
       <c r="J17" s="385" t="inlineStr">
         <is>
@@ -21057,11 +19870,7 @@
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
-      <c r="B18" s="377" t="inlineStr">
-        <is>
-          <t>HV Kademeler</t>
-        </is>
-      </c>
+      <c r="B18" s="377" t="n"/>
       <c r="F18" s="463">
         <f>'ANA SAYFA'!O59</f>
         <v/>
@@ -21095,11 +19904,7 @@
     </row>
     <row r="19" ht="15.75" customHeight="1" s="227">
       <c r="A19" s="10" t="n"/>
-      <c r="B19" s="377" t="inlineStr">
-        <is>
-          <t>LV Ratings</t>
-        </is>
-      </c>
+      <c r="B19" s="377" t="n"/>
       <c r="F19" s="461" t="n">
         <v>231</v>
       </c>
@@ -21135,11 +19940,7 @@
     </row>
     <row r="20" ht="15.75" customHeight="1" s="227">
       <c r="A20" s="10" t="n"/>
-      <c r="B20" s="377" t="inlineStr">
-        <is>
-          <t>Çevirme Oranı</t>
-        </is>
-      </c>
+      <c r="B20" s="377" t="n"/>
       <c r="F20" s="462">
         <f>F18/T15</f>
         <v/>
@@ -22053,7 +20854,7 @@
     <col width="3.5546875" customWidth="1" style="227" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="15" customHeight="1" s="227">
       <c r="A1" s="12" t="n"/>
       <c r="B1" s="13" t="n"/>
       <c r="C1" s="13" t="n"/>
@@ -22135,7 +20936,7 @@
       <c r="Q3" s="213" t="n"/>
       <c r="R3" s="11" t="n"/>
     </row>
-    <row r="4">
+    <row r="4" ht="15" customHeight="1" s="227">
       <c r="A4" s="10" t="n"/>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="127" t="n"/>
@@ -22183,7 +20984,7 @@
       <c r="Q5" s="482" t="n"/>
       <c r="R5" s="11" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" ht="15" customHeight="1" s="227">
       <c r="A6" s="10" t="n"/>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="127" t="n"/>
@@ -22250,7 +21051,7 @@
       <c r="Q8" s="143" t="n"/>
       <c r="R8" s="11" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="15" customHeight="1" s="227">
       <c r="A9" s="10" t="n"/>
       <c r="B9" s="421" t="inlineStr">
         <is>
@@ -22271,11 +21072,7 @@
         </is>
       </c>
       <c r="I9" s="482" t="n"/>
-      <c r="J9" s="374" t="inlineStr">
-        <is>
-          <t>METREL-MI3123</t>
-        </is>
-      </c>
+      <c r="J9" s="374" t="n"/>
       <c r="K9" s="99" t="n"/>
       <c r="L9" s="482" t="n"/>
       <c r="M9" s="374" t="inlineStr">
@@ -22284,9 +21081,7 @@
         </is>
       </c>
       <c r="N9" s="482" t="n"/>
-      <c r="O9" s="374" t="n">
-        <v>16350177</v>
-      </c>
+      <c r="O9" s="374" t="n"/>
       <c r="P9" s="99" t="n"/>
       <c r="Q9" s="482" t="n"/>
       <c r="R9" s="11" t="n"/>
@@ -22399,7 +21194,7 @@
       <c r="Q14" s="143" t="n"/>
       <c r="R14" s="11" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="15" customHeight="1" s="227">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="345" t="n"/>
       <c r="C15" s="99" t="n"/>
@@ -22423,7 +21218,7 @@
       <c r="Q15" s="482" t="n"/>
       <c r="R15" s="11" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="15" customHeight="1" s="227">
       <c r="A16" s="10" t="n"/>
       <c r="B16" s="515" t="inlineStr">
         <is>
@@ -22471,7 +21266,7 @@
       <c r="Q16" s="482" t="n"/>
       <c r="R16" s="11" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="15" customHeight="1" s="227">
       <c r="A17" s="10" t="n"/>
       <c r="B17" s="518" t="n"/>
       <c r="C17" s="519" t="n"/>
@@ -22491,7 +21286,7 @@
       <c r="Q17" s="428" t="n"/>
       <c r="R17" s="11" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" ht="15" customHeight="1" s="227">
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="521" t="n"/>
       <c r="C18" s="45" t="n"/>
@@ -22521,7 +21316,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="15" customHeight="1" s="227">
       <c r="A19" s="10" t="n"/>
       <c r="B19" s="521" t="n"/>
       <c r="C19" s="45" t="n"/>
@@ -22541,7 +21336,7 @@
       <c r="Q19" s="522" t="n"/>
       <c r="R19" s="11" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" ht="15" customHeight="1" s="227">
       <c r="A20" s="10" t="n"/>
       <c r="B20" s="521" t="n"/>
       <c r="C20" s="45" t="n"/>
@@ -22561,7 +21356,7 @@
       <c r="Q20" s="522" t="n"/>
       <c r="R20" s="11" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" ht="15" customHeight="1" s="227">
       <c r="A21" s="10" t="n"/>
       <c r="B21" s="521" t="n"/>
       <c r="C21" s="45" t="n"/>
@@ -22581,7 +21376,7 @@
       <c r="Q21" s="522" t="n"/>
       <c r="R21" s="11" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="15" customHeight="1" s="227">
       <c r="A22" s="10" t="n"/>
       <c r="B22" s="521" t="n"/>
       <c r="C22" s="45" t="n"/>
@@ -22961,7 +21756,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="15" customHeight="1" s="227">
       <c r="A32" s="10" t="n"/>
       <c r="B32" s="3" t="n"/>
       <c r="C32" s="127" t="n"/>
@@ -23031,7 +21826,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="15" customHeight="1" s="227">
       <c r="A35" s="10" t="n"/>
       <c r="B35" s="3" t="n"/>
       <c r="C35" s="127" t="n"/>
@@ -23750,7 +22545,7 @@
       <c r="S10" s="41" t="n"/>
       <c r="T10" s="11" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="15" customHeight="1" s="227">
       <c r="A11" s="10" t="n"/>
       <c r="B11" s="280" t="inlineStr">
         <is>
@@ -23762,11 +22557,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G11" s="542" t="inlineStr">
-        <is>
-          <t>ULUSOY</t>
-        </is>
-      </c>
+      <c r="G11" s="542" t="n"/>
       <c r="H11" s="486" t="n"/>
       <c r="I11" s="486" t="n"/>
       <c r="J11" s="486" t="n"/>
@@ -23780,11 +22571,7 @@
           <t xml:space="preserve">: </t>
         </is>
       </c>
-      <c r="O11" s="543" t="inlineStr">
-        <is>
-          <t>USFB-36R</t>
-        </is>
-      </c>
+      <c r="O11" s="543" t="n"/>
       <c r="P11" s="486" t="n"/>
       <c r="Q11" s="486" t="n"/>
       <c r="R11" s="486" t="n"/>
@@ -23813,7 +22600,7 @@
       <c r="S12" s="547" t="n"/>
       <c r="T12" s="11" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="15" customHeight="1" s="227">
       <c r="A13" s="10" t="n"/>
       <c r="B13" s="247" t="inlineStr">
         <is>
@@ -23825,9 +22612,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G13" s="548" t="n">
-        <v>630</v>
-      </c>
+      <c r="G13" s="548" t="n"/>
       <c r="H13" s="486" t="n"/>
       <c r="I13" s="486" t="n"/>
       <c r="J13" s="486" t="n"/>
@@ -23841,11 +22626,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="O13" s="550" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
-      </c>
+      <c r="O13" s="550" t="n"/>
       <c r="P13" s="486" t="n"/>
       <c r="Q13" s="486" t="n"/>
       <c r="R13" s="486" t="n"/>
@@ -23874,7 +22655,7 @@
       <c r="S14" s="547" t="n"/>
       <c r="T14" s="11" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="15" customHeight="1" s="227">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="280" t="inlineStr">
         <is>
@@ -23886,9 +22667,7 @@
           <t xml:space="preserve">:  </t>
         </is>
       </c>
-      <c r="G15" s="548" t="n">
-        <v>36000</v>
-      </c>
+      <c r="G15" s="548" t="n"/>
       <c r="H15" s="486" t="n"/>
       <c r="I15" s="486" t="n"/>
       <c r="J15" s="486" t="n"/>
@@ -23902,9 +22681,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="O15" s="551" t="n">
-        <v>2196</v>
-      </c>
+      <c r="O15" s="551" t="n"/>
       <c r="P15" s="486" t="n"/>
       <c r="Q15" s="486" t="n"/>
       <c r="R15" s="486" t="n"/>
@@ -23945,11 +22722,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G17" s="548" t="inlineStr">
-        <is>
-          <t>220 Vac</t>
-        </is>
-      </c>
+      <c r="G17" s="548" t="n"/>
       <c r="H17" s="486" t="n"/>
       <c r="I17" s="486" t="n"/>
       <c r="J17" s="486" t="n"/>
@@ -23963,11 +22736,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="O17" s="551" t="inlineStr">
-        <is>
-          <t>24 Vdc</t>
-        </is>
-      </c>
+      <c r="O17" s="551" t="n"/>
       <c r="P17" s="486" t="n"/>
       <c r="Q17" s="486" t="n"/>
       <c r="R17" s="486" t="n"/>
@@ -24126,7 +22895,7 @@
       <c r="S23" s="143" t="n"/>
       <c r="T23" s="11" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" ht="15" customHeight="1" s="227">
       <c r="A24" s="10" t="n"/>
       <c r="B24" s="280" t="inlineStr">
         <is>
@@ -24138,17 +22907,9 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G24" s="552" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="G24" s="552" t="n"/>
       <c r="H24" s="487" t="n"/>
-      <c r="I24" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="I24" s="553" t="n"/>
       <c r="J24" s="554" t="n"/>
       <c r="K24" s="291" t="inlineStr">
         <is>
@@ -24160,17 +22921,9 @@
           <t>:</t>
         </is>
       </c>
-      <c r="P24" s="552" t="inlineStr">
-        <is>
-          <t>YAPILDI</t>
-        </is>
-      </c>
+      <c r="P24" s="552" t="n"/>
       <c r="Q24" s="487" t="n"/>
-      <c r="R24" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="R24" s="553" t="n"/>
       <c r="S24" s="554" t="n"/>
       <c r="T24" s="11" t="n"/>
     </row>
@@ -24196,7 +22949,7 @@
       <c r="S25" s="120" t="n"/>
       <c r="T25" s="11" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" ht="15" customHeight="1" s="227">
       <c r="A26" s="10" t="n"/>
       <c r="B26" s="280" t="inlineStr">
         <is>
@@ -24208,19 +22961,9 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G26" s="557" t="n">
-        <v>24</v>
-      </c>
-      <c r="H26" s="552" t="inlineStr">
-        <is>
-          <t>Vdc</t>
-        </is>
-      </c>
-      <c r="I26" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="G26" s="557" t="n"/>
+      <c r="H26" s="552" t="n"/>
+      <c r="I26" s="553" t="n"/>
       <c r="J26" s="554" t="n"/>
       <c r="K26" s="291" t="inlineStr">
         <is>
@@ -24232,17 +22975,9 @@
           <t>:</t>
         </is>
       </c>
-      <c r="P26" s="552" t="inlineStr">
-        <is>
-          <t>YAPILDI</t>
-        </is>
-      </c>
+      <c r="P26" s="552" t="n"/>
       <c r="Q26" s="487" t="n"/>
-      <c r="R26" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="R26" s="553" t="n"/>
       <c r="S26" s="554" t="n"/>
       <c r="T26" s="11" t="n"/>
     </row>
@@ -24268,7 +23003,7 @@
       <c r="S27" s="120" t="n"/>
       <c r="T27" s="11" t="n"/>
     </row>
-    <row r="28">
+    <row r="28" ht="15" customHeight="1" s="227">
       <c r="A28" s="10" t="n"/>
       <c r="B28" s="280" t="inlineStr">
         <is>
@@ -24280,17 +23015,9 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G28" s="552" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="G28" s="552" t="n"/>
       <c r="H28" s="487" t="n"/>
-      <c r="I28" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="I28" s="553" t="n"/>
       <c r="J28" s="93" t="n"/>
       <c r="K28" s="291" t="inlineStr">
         <is>
@@ -24302,17 +23029,9 @@
           <t xml:space="preserve">: </t>
         </is>
       </c>
-      <c r="P28" s="552" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="P28" s="552" t="n"/>
       <c r="Q28" s="487" t="n"/>
-      <c r="R28" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="R28" s="553" t="n"/>
       <c r="S28" s="93" t="n"/>
       <c r="T28" s="11" t="n"/>
     </row>
@@ -24338,7 +23057,7 @@
       <c r="S29" s="120" t="n"/>
       <c r="T29" s="11" t="n"/>
     </row>
-    <row r="30">
+    <row r="30" ht="15" customHeight="1" s="227">
       <c r="A30" s="10" t="n"/>
       <c r="B30" s="280" t="inlineStr">
         <is>
@@ -24350,17 +23069,9 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G30" s="552" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="G30" s="552" t="n"/>
       <c r="H30" s="487" t="n"/>
-      <c r="I30" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="I30" s="553" t="n"/>
       <c r="J30" s="93" t="n"/>
       <c r="K30" s="291" t="inlineStr">
         <is>
@@ -24372,17 +23083,9 @@
           <t>:</t>
         </is>
       </c>
-      <c r="P30" s="552" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="P30" s="552" t="n"/>
       <c r="Q30" s="487" t="n"/>
-      <c r="R30" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="R30" s="553" t="n"/>
       <c r="S30" s="93" t="n"/>
       <c r="T30" s="11" t="n"/>
     </row>
@@ -24408,7 +23111,7 @@
       <c r="S31" s="120" t="n"/>
       <c r="T31" s="11" t="n"/>
     </row>
-    <row r="32">
+    <row r="32" ht="15" customHeight="1" s="227">
       <c r="A32" s="10" t="n"/>
       <c r="B32" s="280" t="inlineStr">
         <is>
@@ -24420,17 +23123,9 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G32" s="552" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="G32" s="552" t="n"/>
       <c r="H32" s="487" t="n"/>
-      <c r="I32" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="I32" s="553" t="n"/>
       <c r="J32" s="93" t="n"/>
       <c r="K32" s="291" t="inlineStr">
         <is>
@@ -24442,17 +23137,9 @@
           <t>:</t>
         </is>
       </c>
-      <c r="P32" s="552" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="P32" s="552" t="n"/>
       <c r="Q32" s="487" t="n"/>
-      <c r="R32" s="553" t="inlineStr">
-        <is>
-          <t>ü</t>
-        </is>
-      </c>
+      <c r="R32" s="553" t="n"/>
       <c r="S32" s="93" t="n"/>
       <c r="T32" s="11" t="n"/>
     </row>
@@ -25027,11 +23714,7 @@
           <t>L-1</t>
         </is>
       </c>
-      <c r="C50" s="561" t="inlineStr">
-        <is>
-          <t>10.00</t>
-        </is>
-      </c>
+      <c r="C50" s="561" t="n"/>
       <c r="D50" s="99" t="n"/>
       <c r="E50" s="99" t="n"/>
       <c r="F50" s="562" t="inlineStr">
@@ -25039,9 +23722,7 @@
           <t>kV</t>
         </is>
       </c>
-      <c r="G50" s="563" t="n">
-        <v>20000</v>
-      </c>
+      <c r="G50" s="563" t="n"/>
       <c r="H50" s="99" t="n"/>
       <c r="I50" s="564" t="inlineStr">
         <is>
@@ -25052,17 +23733,11 @@
         <f>IF(G50&gt;50,1,0)</f>
         <v/>
       </c>
-      <c r="K50" s="376" t="inlineStr">
-        <is>
-          <t>80.00A</t>
-        </is>
-      </c>
+      <c r="K50" s="376" t="n"/>
       <c r="L50" s="99" t="n"/>
       <c r="M50" s="99" t="n"/>
       <c r="N50" s="482" t="n"/>
-      <c r="O50" s="566" t="n">
-        <v>110</v>
-      </c>
+      <c r="O50" s="566" t="n"/>
       <c r="P50" s="99" t="n"/>
       <c r="Q50" s="99" t="n"/>
       <c r="R50" s="564" t="inlineStr">
@@ -25143,11 +23818,7 @@
           <t>L-2</t>
         </is>
       </c>
-      <c r="C52" s="561" t="inlineStr">
-        <is>
-          <t>10.00</t>
-        </is>
-      </c>
+      <c r="C52" s="561" t="n"/>
       <c r="D52" s="99" t="n"/>
       <c r="E52" s="99" t="n"/>
       <c r="F52" s="562" t="inlineStr">
@@ -25155,9 +23826,7 @@
           <t>kV</t>
         </is>
       </c>
-      <c r="G52" s="563" t="n">
-        <v>20000</v>
-      </c>
+      <c r="G52" s="563" t="n"/>
       <c r="H52" s="99" t="n"/>
       <c r="I52" s="564" t="inlineStr">
         <is>
@@ -25168,17 +23837,11 @@
         <f>IF(G52&gt;50,1,0)</f>
         <v/>
       </c>
-      <c r="K52" s="376" t="inlineStr">
-        <is>
-          <t>80.00A</t>
-        </is>
-      </c>
+      <c r="K52" s="376" t="n"/>
       <c r="L52" s="99" t="n"/>
       <c r="M52" s="99" t="n"/>
       <c r="N52" s="482" t="n"/>
-      <c r="O52" s="571" t="n">
-        <v>40</v>
-      </c>
+      <c r="O52" s="571" t="n"/>
       <c r="P52" s="99" t="n"/>
       <c r="Q52" s="99" t="n"/>
       <c r="R52" s="564" t="inlineStr">
@@ -25259,11 +23922,7 @@
           <t>L-3</t>
         </is>
       </c>
-      <c r="C54" s="561" t="inlineStr">
-        <is>
-          <t>10.00</t>
-        </is>
-      </c>
+      <c r="C54" s="561" t="n"/>
       <c r="D54" s="99" t="n"/>
       <c r="E54" s="99" t="n"/>
       <c r="F54" s="562" t="inlineStr">
@@ -25271,9 +23930,7 @@
           <t>kV</t>
         </is>
       </c>
-      <c r="G54" s="563" t="n">
-        <v>20000</v>
-      </c>
+      <c r="G54" s="563" t="n"/>
       <c r="H54" s="99" t="n"/>
       <c r="I54" s="564" t="inlineStr">
         <is>
@@ -25284,17 +23941,11 @@
         <f>IF(G54&gt;50,1,0)</f>
         <v/>
       </c>
-      <c r="K54" s="376" t="inlineStr">
-        <is>
-          <t>80.00A</t>
-        </is>
-      </c>
+      <c r="K54" s="376" t="n"/>
       <c r="L54" s="99" t="n"/>
       <c r="M54" s="99" t="n"/>
       <c r="N54" s="482" t="n"/>
-      <c r="O54" s="571" t="n">
-        <v>54</v>
-      </c>
+      <c r="O54" s="571" t="n"/>
       <c r="P54" s="99" t="n"/>
       <c r="Q54" s="99" t="n"/>
       <c r="R54" s="564" t="inlineStr">
@@ -25588,9 +24239,7 @@
           <t>L-1</t>
         </is>
       </c>
-      <c r="C61" s="572" t="n">
-        <v>75.34999999999999</v>
-      </c>
+      <c r="C61" s="572" t="n"/>
       <c r="D61" s="99" t="n"/>
       <c r="E61" s="482" t="inlineStr">
         <is>
@@ -25608,9 +24257,7 @@
         </is>
       </c>
       <c r="I61" s="482" t="n"/>
-      <c r="J61" s="572" t="n">
-        <v>69.03</v>
-      </c>
+      <c r="J61" s="572" t="n"/>
       <c r="K61" s="99" t="n"/>
       <c r="L61" s="482" t="inlineStr">
         <is>
@@ -25628,11 +24275,7 @@
         </is>
       </c>
       <c r="P61" s="482" t="n"/>
-      <c r="Q61" s="573" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="Q61" s="573" t="n"/>
       <c r="R61" s="99" t="n"/>
       <c r="S61" s="482" t="n"/>
       <c r="T61" s="11" t="n"/>
@@ -25700,9 +24343,7 @@
           <t>L-2</t>
         </is>
       </c>
-      <c r="C63" s="572" t="n">
-        <v>74.98</v>
-      </c>
+      <c r="C63" s="572" t="n"/>
       <c r="D63" s="99" t="n"/>
       <c r="E63" s="482" t="inlineStr">
         <is>
@@ -25717,9 +24358,7 @@
       <c r="G63" s="99" t="n"/>
       <c r="H63" s="99" t="n"/>
       <c r="I63" s="482" t="n"/>
-      <c r="J63" s="572" t="n">
-        <v>66.56999999999999</v>
-      </c>
+      <c r="J63" s="572" t="n"/>
       <c r="K63" s="99" t="n"/>
       <c r="L63" s="482" t="inlineStr">
         <is>
@@ -25734,11 +24373,7 @@
       <c r="N63" s="99" t="n"/>
       <c r="O63" s="99" t="n"/>
       <c r="P63" s="482" t="n"/>
-      <c r="Q63" s="573" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="Q63" s="573" t="n"/>
       <c r="R63" s="99" t="n"/>
       <c r="S63" s="482" t="n"/>
       <c r="T63" s="11" t="n"/>
@@ -25780,25 +24415,21 @@
       <c r="S64" s="212" t="n"/>
       <c r="T64" s="11" t="n"/>
     </row>
-    <row r="65">
+    <row r="65" ht="15" customHeight="1" s="227">
       <c r="A65" s="10" t="n"/>
       <c r="B65" s="504" t="inlineStr">
         <is>
           <t>L-3</t>
         </is>
       </c>
-      <c r="C65" s="572" t="n">
-        <v>75.15000000000001</v>
-      </c>
+      <c r="C65" s="572" t="n"/>
       <c r="D65" s="99" t="n"/>
       <c r="E65" s="482" t="inlineStr">
         <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="F65" s="576" t="n">
-        <v>2.6</v>
-      </c>
+      <c r="F65" s="576" t="n"/>
       <c r="G65" s="99" t="n"/>
       <c r="H65" s="398" t="inlineStr">
         <is>
@@ -25806,18 +24437,14 @@
         </is>
       </c>
       <c r="I65" s="482" t="n"/>
-      <c r="J65" s="572" t="n">
-        <v>68.79000000000001</v>
-      </c>
+      <c r="J65" s="572" t="n"/>
       <c r="K65" s="99" t="n"/>
       <c r="L65" s="482" t="inlineStr">
         <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="M65" s="576" t="n">
-        <v>1.3</v>
-      </c>
+      <c r="M65" s="576" t="n"/>
       <c r="N65" s="99" t="n"/>
       <c r="O65" s="398" t="inlineStr">
         <is>
@@ -25825,11 +24452,7 @@
         </is>
       </c>
       <c r="P65" s="482" t="n"/>
-      <c r="Q65" s="573" t="inlineStr">
-        <is>
-          <t>UYGUN</t>
-        </is>
-      </c>
+      <c r="Q65" s="573" t="n"/>
       <c r="R65" s="99" t="n"/>
       <c r="S65" s="482" t="n"/>
       <c r="T65" s="11" t="n"/>
@@ -26128,9 +24751,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F77" s="596" t="n">
-        <v>88258</v>
-      </c>
+      <c r="F77" s="596" t="n"/>
       <c r="J77" s="212" t="n"/>
       <c r="K77" s="267" t="n"/>
       <c r="L77" s="277" t="n"/>
@@ -26157,11 +24778,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F78" s="600" t="inlineStr">
-        <is>
-          <t>K202439698</t>
-        </is>
-      </c>
+      <c r="F78" s="600" t="n"/>
       <c r="G78" s="50" t="n"/>
       <c r="H78" s="50" t="n"/>
       <c r="I78" s="50" t="n"/>
@@ -26199,7 +24816,7 @@
       <c r="S79" s="16" t="n"/>
       <c r="T79" s="17" t="n"/>
     </row>
-    <row r="80">
+    <row r="80" ht="15" customHeight="1" s="227">
       <c r="V80" s="602">
         <f>C61-C63</f>
         <v/>
@@ -26209,7 +24826,7 @@
         <v/>
       </c>
     </row>
-    <row r="81">
+    <row r="81" ht="15" customHeight="1" s="227">
       <c r="V81" s="602">
         <f>C61-C65</f>
         <v/>
@@ -26219,7 +24836,7 @@
         <v/>
       </c>
     </row>
-    <row r="82">
+    <row r="82" ht="15" customHeight="1" s="227">
       <c r="V82" s="602">
         <f>C63-C65</f>
         <v/>
@@ -26229,7 +24846,7 @@
         <v/>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="15" customHeight="1" s="227">
       <c r="V83" s="602">
         <f>C63-C61</f>
         <v/>
@@ -26239,7 +24856,7 @@
         <v/>
       </c>
     </row>
-    <row r="84">
+    <row r="84" ht="15" customHeight="1" s="227">
       <c r="V84" s="602">
         <f>C65-C61</f>
         <v/>
@@ -26249,7 +24866,7 @@
         <v/>
       </c>
     </row>
-    <row r="85">
+    <row r="85" ht="15" customHeight="1" s="227">
       <c r="V85" s="602">
         <f>C65-C63</f>
         <v/>
@@ -26388,7 +25005,7 @@
     <col width="9.109375" customWidth="1" style="227" min="19" max="19"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="15" customHeight="1" s="227">
       <c r="A1" s="12" t="n"/>
       <c r="B1" s="13" t="n"/>
       <c r="C1" s="13" t="n"/>
@@ -26601,7 +25218,7 @@
       <c r="Q9" s="143" t="n"/>
       <c r="R9" s="11" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="15" customHeight="1" s="227">
       <c r="A10" s="10" t="n"/>
       <c r="B10" s="421" t="inlineStr">
         <is>
@@ -26609,11 +25226,7 @@
         </is>
       </c>
       <c r="C10" s="482" t="n"/>
-      <c r="D10" s="422" t="inlineStr">
-        <is>
-          <t>Hilmi GÜL</t>
-        </is>
-      </c>
+      <c r="D10" s="422" t="n"/>
       <c r="E10" s="99" t="n"/>
       <c r="F10" s="99" t="n"/>
       <c r="G10" s="482" t="n"/>
@@ -26623,11 +25236,7 @@
         </is>
       </c>
       <c r="I10" s="482" t="n"/>
-      <c r="J10" s="374" t="inlineStr">
-        <is>
-          <t>METREL MI 3210</t>
-        </is>
-      </c>
+      <c r="J10" s="374" t="n"/>
       <c r="K10" s="99" t="n"/>
       <c r="L10" s="482" t="n"/>
       <c r="M10" s="374" t="inlineStr">
@@ -26636,9 +25245,7 @@
         </is>
       </c>
       <c r="N10" s="482" t="n"/>
-      <c r="O10" s="374" t="n">
-        <v>16060016</v>
-      </c>
+      <c r="O10" s="374" t="n"/>
       <c r="P10" s="99" t="n"/>
       <c r="Q10" s="482" t="n"/>
       <c r="R10" s="11" t="n"/>
@@ -26771,7 +25378,7 @@
       <c r="Q15" s="143" t="n"/>
       <c r="R15" s="11" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="15" customHeight="1" s="227">
       <c r="A16" s="10" t="n"/>
       <c r="B16" s="345" t="inlineStr">
         <is>
@@ -26813,7 +25420,7 @@
       <c r="Q16" s="482" t="n"/>
       <c r="R16" s="11" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="15" customHeight="1" s="227">
       <c r="A17" s="10" t="n"/>
       <c r="B17" s="515" t="inlineStr">
         <is>
@@ -26863,7 +25470,7 @@
       <c r="Q17" s="482" t="n"/>
       <c r="R17" s="11" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" ht="15" customHeight="1" s="227">
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="515" t="inlineStr">
         <is>
@@ -26913,7 +25520,7 @@
       <c r="Q18" s="482" t="n"/>
       <c r="R18" s="11" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="15" customHeight="1" s="227">
       <c r="A19" s="10" t="n"/>
       <c r="B19" s="515" t="inlineStr">
         <is>
@@ -26963,7 +25570,7 @@
       <c r="Q19" s="482" t="n"/>
       <c r="R19" s="11" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" ht="15" customHeight="1" s="227">
       <c r="A20" s="33" t="n"/>
       <c r="Q20" s="211" t="n"/>
       <c r="R20" s="11" t="n"/>
@@ -26972,22 +25579,22 @@
         <v/>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="15" customHeight="1" s="227">
       <c r="A21" s="33" t="n"/>
       <c r="Q21" s="212" t="n"/>
       <c r="R21" s="11" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="15" customHeight="1" s="227">
       <c r="A22" s="33" t="n"/>
       <c r="Q22" s="212" t="n"/>
       <c r="R22" s="11" t="n"/>
     </row>
-    <row r="23">
+    <row r="23" ht="15" customHeight="1" s="227">
       <c r="A23" s="33" t="n"/>
       <c r="Q23" s="212" t="n"/>
       <c r="R23" s="11" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" ht="15" customHeight="1" s="227">
       <c r="A24" s="33" t="n"/>
       <c r="Q24" s="212" t="n"/>
       <c r="R24" s="11" t="n"/>
@@ -26996,17 +25603,17 @@
         <v/>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="15" customHeight="1" s="227">
       <c r="A25" s="33" t="n"/>
       <c r="Q25" s="212" t="n"/>
       <c r="R25" s="11" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" ht="15" customHeight="1" s="227">
       <c r="A26" s="33" t="n"/>
       <c r="Q26" s="212" t="n"/>
       <c r="R26" s="11" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="15" customHeight="1" s="227">
       <c r="A27" s="33" t="n"/>
       <c r="Q27" s="212" t="n"/>
       <c r="R27" s="11" t="n"/>
@@ -27016,7 +25623,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="15" customHeight="1" s="227">
       <c r="A28" s="33" t="n"/>
       <c r="Q28" s="212" t="n"/>
       <c r="R28" s="11" t="n"/>
@@ -27035,7 +25642,7 @@
       <c r="A30" s="10" t="n"/>
       <c r="R30" s="11" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" ht="15" customHeight="1" s="227">
       <c r="A31" s="10" t="n"/>
       <c r="R31" s="11" t="n"/>
     </row>
@@ -27059,7 +25666,7 @@
       <c r="A36" s="10" t="n"/>
       <c r="R36" s="11" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" ht="15" customHeight="1" s="227">
       <c r="A37" s="10" t="n"/>
       <c r="B37" s="3" t="n"/>
       <c r="C37" s="317" t="n"/>
@@ -27079,7 +25686,7 @@
       <c r="Q37" s="117" t="n"/>
       <c r="R37" s="11" t="n"/>
     </row>
-    <row r="38">
+    <row r="38" ht="15" customHeight="1" s="227">
       <c r="A38" s="10" t="n"/>
       <c r="B38" s="528" t="n"/>
       <c r="C38" s="317" t="n"/>
@@ -27093,7 +25700,7 @@
       <c r="Q38" s="143" t="n"/>
       <c r="R38" s="11" t="n"/>
     </row>
-    <row r="39">
+    <row r="39" ht="15" customHeight="1" s="227">
       <c r="A39" s="10" t="n"/>
       <c r="B39" s="528" t="n"/>
       <c r="C39" s="317" t="n"/>
@@ -27113,7 +25720,7 @@
       <c r="Q39" s="143" t="n"/>
       <c r="R39" s="11" t="n"/>
     </row>
-    <row r="40">
+    <row r="40" ht="15" customHeight="1" s="227">
       <c r="A40" s="10" t="n"/>
       <c r="B40" s="528" t="n"/>
       <c r="C40" s="317" t="n"/>
@@ -27127,7 +25734,7 @@
       <c r="Q40" s="143" t="n"/>
       <c r="R40" s="11" t="n"/>
     </row>
-    <row r="41">
+    <row r="41" ht="15" customHeight="1" s="227">
       <c r="A41" s="10" t="n"/>
       <c r="B41" s="528" t="n"/>
       <c r="C41" s="317" t="n"/>
@@ -27147,7 +25754,7 @@
       <c r="Q41" s="143" t="n"/>
       <c r="R41" s="11" t="n"/>
     </row>
-    <row r="42">
+    <row r="42" ht="15" customHeight="1" s="227">
       <c r="A42" s="10" t="n"/>
       <c r="B42" s="528" t="n"/>
       <c r="C42" s="317" t="n"/>
@@ -27167,7 +25774,7 @@
       <c r="Q42" s="143" t="n"/>
       <c r="R42" s="11" t="n"/>
     </row>
-    <row r="43">
+    <row r="43" ht="15" customHeight="1" s="227">
       <c r="A43" s="10" t="n"/>
       <c r="B43" s="528" t="n"/>
       <c r="C43" s="317" t="n"/>
@@ -27187,7 +25794,7 @@
       <c r="Q43" s="143" t="n"/>
       <c r="R43" s="11" t="n"/>
     </row>
-    <row r="44">
+    <row r="44" ht="15" customHeight="1" s="227">
       <c r="A44" s="10" t="n"/>
       <c r="B44" s="528" t="n"/>
       <c r="C44" s="317" t="n"/>
@@ -27207,7 +25814,7 @@
       <c r="Q44" s="143" t="n"/>
       <c r="R44" s="11" t="n"/>
     </row>
-    <row r="45">
+    <row r="45" ht="15" customHeight="1" s="227">
       <c r="A45" s="10" t="n"/>
       <c r="B45" s="528" t="n"/>
       <c r="C45" s="317" t="n"/>
@@ -27227,7 +25834,7 @@
       <c r="Q45" s="143" t="n"/>
       <c r="R45" s="11" t="n"/>
     </row>
-    <row r="46">
+    <row r="46" ht="15" customHeight="1" s="227">
       <c r="A46" s="10" t="n"/>
       <c r="B46" s="118" t="n"/>
       <c r="C46" s="23" t="n"/>
@@ -27443,6 +26050,7 @@
     <mergeCell ref="J8:Q8"/>
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="B16:C16"/>
+    <mergeCell ref="K18:L18"/>
     <mergeCell ref="X28:AF28"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="D19:E19"/>
@@ -27499,14 +26107,13 @@
     <mergeCell ref="J10:L10"/>
     <mergeCell ref="O18:Q18"/>
     <mergeCell ref="B2:F3"/>
-    <mergeCell ref="I40:J40"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="O38:P38"/>
     <mergeCell ref="K19:L19"/>
     <mergeCell ref="B52:D52"/>
     <mergeCell ref="G40:H40"/>
     <mergeCell ref="K2:Q2"/>
-    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="I40:J40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>